<commit_message>
Import Acute Care (EN) into the content-landing template
- parsers/columns.js: AEM text-image teasers -> Columns block, one row of
  [text | image] or [image | text] in source order (catalog variants
  v_37fdc84c086b, v_6defe37a8d19)
- import-content-landing.js: columns parser and selectors (excludes hero and
  card-grid teasers); acutecare URL added; bundle rebuilt
- myastrazeneca-cleanup.js: drop the login-only Social Features widget
  (anonymous placeholders 'errorMessage requestToSignInContent')
- page-templates.json: acutecare URL and columns mapping

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-landing.report.xlsx
+++ b/tools/importer/reports/import-content-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>_reportFile</t>
   </si>
@@ -59,6 +59,24 @@
   </si>
   <si>
     <t>https://www.myastrazeneca.ch/en/startseite.html</t>
+  </si>
+  <si>
+    <t>en/startseite/therapiegebiete/cvrm/acutecare.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark-withimg","cards-light-withimg","columns","columns","columns","columns"]</t>
+  </si>
+  <si>
+    <t>en/startseite/therapiegebiete/cvrm/acutecare</t>
+  </si>
+  <si>
+    <t>2026-09-30T04:38:24.621Z</t>
+  </si>
+  <si>
+    <t>Acute Care</t>
+  </si>
+  <si>
+    <t>https://www.myastrazeneca.ch/en/startseite/therapiegebiete/cvrm/acutecare.html</t>
   </si>
 </sst>
 </file>
@@ -447,16 +465,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="49" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +526,32 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cards: fold the cards-light-withimg fork into cards as the light variant
- blocks/cards: each card's layout follows the authored content (an
  image-only cell becomes the card image; text-only cards work). Variant
  `light` ("Cards (Light)") carries the oneAZ light card grid from the fork:
  light surface, border, Mulberry titles, Magenta links, 3:2 images,
  1/2/3 columns
- blocks/cards-light-withimg: reduced to a deprecated alias that runs
  cards + light, so the 11 live pages keep rendering until re-published;
  measured identical to the live fork (columns, gap, surface, border, image
  ratio, padding, title and link colours)
- Importer: parsers/cards.js emits "Cards (light)"; 11 EN pages re-imported
  (now Hero (Minimal Dark) + Cards (Light), no old block names)
- Block library demo, blocks.json, block-mapping.json (cards variants ->
  cards; the 3-up grid -> light), README and report updated

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-landing.report.xlsx
+++ b/tools/importer/reports/import-content-landing.report.xlsx
@@ -40,7 +40,7 @@
     <t>en/startseite.report.json</t>
   </si>
   <si>
-    <t>["hero","cards-light-withimg","columns"]</t>
+    <t>["hero","cards","columns"]</t>
   </si>
   <si>
     <t>en/startseite</t>
@@ -52,7 +52,7 @@
     <t>content-landing</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:13.583Z</t>
+    <t>2026-10-01T08:37:52.250Z</t>
   </si>
   <si>
     <t>Home | MyAstraZeneca</t>
@@ -64,13 +64,13 @@
     <t>en/startseite/therapiegebiete/cvrm/acutecare.report.json</t>
   </si>
   <si>
-    <t>["hero","cards-light-withimg","columns","columns","columns","columns"]</t>
+    <t>["hero","cards","columns","columns","columns","columns"]</t>
   </si>
   <si>
     <t>en/startseite/therapiegebiete/cvrm/acutecare</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:18.618Z</t>
+    <t>2026-10-01T08:37:58.526Z</t>
   </si>
   <si>
     <t>Acute Care</t>
@@ -85,7 +85,7 @@
     <t>en/startseite/therapiegebiete/cvrm/chronischeniereninsuffizienz</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:24.521Z</t>
+    <t>2026-10-01T08:38:06.548Z</t>
   </si>
   <si>
     <t>Chronic Kidney Disease (CKD) - Symptoms, Diagnosis &amp; Treatment</t>
@@ -100,7 +100,7 @@
     <t>en/startseite/therapiegebiete/cvrm/diabetes</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:31.743Z</t>
+    <t>2026-10-01T08:38:13.754Z</t>
   </si>
   <si>
     <t>Diabetes</t>
@@ -115,7 +115,7 @@
     <t>en/startseite/therapiegebiete/cvrm/herzinsuffizienz</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:37.532Z</t>
+    <t>2026-10-01T08:38:20.669Z</t>
   </si>
   <si>
     <t>Heart Failure Overview: Symptoms &amp; Treatment</t>
@@ -127,13 +127,13 @@
     <t>en/startseite/therapiegebiete/onkologie/brustkrebs.report.json</t>
   </si>
   <si>
-    <t>["hero","cards-light-withimg","columns","columns","columns"]</t>
+    <t>["hero","cards","columns","columns","columns"]</t>
   </si>
   <si>
     <t>en/startseite/therapiegebiete/onkologie/brustkrebs</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:44.177Z</t>
+    <t>2026-10-01T08:38:25.770Z</t>
   </si>
   <si>
     <t>Breast Cancer Overview: Causes, Symptoms &amp; Therapy</t>
@@ -148,7 +148,7 @@
     <t>en/startseite/therapiegebiete/onkologie/eierstockkrebs</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:48.936Z</t>
+    <t>2026-10-01T08:38:32.396Z</t>
   </si>
   <si>
     <t>Ovarian Cancer Overview: Symptoms &amp; Treatment</t>
@@ -163,7 +163,7 @@
     <t>en/startseite/therapiegebiete/onkologie/lungenkrebs</t>
   </si>
   <si>
-    <t>2026-10-01T08:25:55.218Z</t>
+    <t>2026-10-01T08:38:38.372Z</t>
   </si>
   <si>
     <t>Lung Cancer: Symptoms, Stages &amp; Treatment</t>
@@ -178,7 +178,7 @@
     <t>en/startseite/therapiegebiete/ri/asthma</t>
   </si>
   <si>
-    <t>2026-10-01T08:26:01.077Z</t>
+    <t>2026-10-01T08:38:43.888Z</t>
   </si>
   <si>
     <t>Asthma – Advances in Diagnosis and Care</t>
@@ -190,13 +190,13 @@
     <t>en/startseite/therapiegebiete/ri/copd.report.json</t>
   </si>
   <si>
-    <t>["in-page-nav","accordion","hero","cards-light-withimg","cards-light-withimg","cards-light-withimg","columns","columns","columns","columns"]</t>
+    <t>["in-page-nav","accordion","hero","cards","cards","cards","columns","columns","columns","columns"]</t>
   </si>
   <si>
     <t>en/startseite/therapiegebiete/ri/copd</t>
   </si>
   <si>
-    <t>2026-10-01T08:26:08.327Z</t>
+    <t>2026-10-01T08:38:52.121Z</t>
   </si>
   <si>
     <t>COPD - Symptoms, diagnosis and treatment</t>
@@ -211,7 +211,7 @@
     <t>en/startseite/therapiegebiete/ri/lupus</t>
   </si>
   <si>
-    <t>2026-10-01T08:26:14.314Z</t>
+    <t>2026-10-01T08:38:58.272Z</t>
   </si>
   <si>
     <t>Lupus Insights and Treatment Guidance – For HCPs</t>

</xml_diff>